<commit_message>
se agrego la hoja de comparacion de proyectos en el excel de esp32 y android
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2.74</v>
+        <v>2.77</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>44.69</v>
+        <v>44.6</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>74.11</v>
+        <v>74.23</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1.89</v>
+        <v>1.95</v>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="C12" t="n">
-        <v>634</v>
+        <v>674</v>
       </c>
       <c r="D12" t="n">
-        <v>2.74</v>
+        <v>2.77</v>
       </c>
       <c r="E12" t="n">
-        <v>3063</v>
+        <v>3260</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>13.26</v>
+        <v>13.42</v>
       </c>
     </row>
   </sheetData>
@@ -3415,16 +3415,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3063</v>
+        <v>3260</v>
       </c>
       <c r="C12" t="n">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="D12" t="n">
-        <v>21182</v>
+        <v>22509</v>
       </c>
       <c r="E12" t="n">
-        <v>44.69</v>
+        <v>44.6</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4039,13 +4039,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="D12" t="n">
-        <v>74.11</v>
+        <v>74.23</v>
       </c>
       <c r="E12" t="n">
-        <v>1.89</v>
+        <v>1.95</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4063,17 +4063,17 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="J12" t="n">
         <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>missing-function-docstring: 39; trailing-whitespace: 21; no-member: 16; broad-exception-caught: 11; unused-import: 9; unexpected-keyword-arg: 9; 6/5: 8; 104/100: 7; undefined-variable: 6; protected-access: 5</t>
+          <t>missing-function-docstring: 39; trailing-whitespace: 26; no-member: 16; unexpected-keyword-arg: 16; broad-exception-caught: 11; 6/5: 10; 104/100: 7; unused-import: 6; undefined-variable: 6; protected-access: 5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se realizo la busqueda de proyectos para comparar en la hoja comparacion segun el codigo del proyecto y el dispostivo
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2.77</v>
+        <v>2.81</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>44.6</v>
+        <v>44.55</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>74.23</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C12" t="n">
-        <v>674</v>
+        <v>686</v>
       </c>
       <c r="D12" t="n">
-        <v>2.77</v>
+        <v>2.81</v>
       </c>
       <c r="E12" t="n">
-        <v>3260</v>
+        <v>3365</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>13.42</v>
+        <v>13.79</v>
       </c>
     </row>
   </sheetData>
@@ -3415,16 +3415,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3260</v>
+        <v>3365</v>
       </c>
       <c r="C12" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D12" t="n">
-        <v>22509</v>
+        <v>22877</v>
       </c>
       <c r="E12" t="n">
-        <v>44.6</v>
+        <v>44.55</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4039,13 +4039,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D12" t="n">
-        <v>74.23</v>
+        <v>71.31999999999999</v>
       </c>
       <c r="E12" t="n">
-        <v>1.95</v>
+        <v>1.97</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4063,17 +4063,17 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="J12" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="K12" t="n">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>missing-function-docstring: 39; trailing-whitespace: 26; no-member: 16; unexpected-keyword-arg: 16; broad-exception-caught: 11; 6/5: 10; 104/100: 7; unused-import: 6; undefined-variable: 6; protected-access: 5</t>
+          <t>missing-function-docstring: 39; trailing-whitespace: 26; no-member: 16; unexpected-keyword-arg: 16; broad-exception-caught: 11; 6/5: 10; 104/100: 7; undefined-variable: 6; protected-access: 5; 106/100: 4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
se genero la hoja que de graficos comparativos en el excel resultante de esp32 y android
</commit_message>
<xml_diff>
--- a/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
+++ b/medidor de metricas/automatizacion_completa/metricas_resultados_pc.xlsx
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="F12" s="4" t="n">
-        <v>2.81</v>
+        <v>2.84</v>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
@@ -2581,7 +2581,7 @@
         </is>
       </c>
       <c r="H12" s="4" t="n">
-        <v>44.55</v>
+        <v>43.94</v>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
@@ -2589,10 +2589,10 @@
         </is>
       </c>
       <c r="J12" s="4" t="n">
-        <v>71.31999999999999</v>
+        <v>72.26000000000001</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>1.97</v>
+        <v>1.93</v>
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
@@ -3033,16 +3033,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="C12" t="n">
-        <v>686</v>
+        <v>701</v>
       </c>
       <c r="D12" t="n">
-        <v>2.81</v>
+        <v>2.84</v>
       </c>
       <c r="E12" t="n">
-        <v>3365</v>
+        <v>3432</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -3055,7 +3055,7 @@
         </is>
       </c>
       <c r="H12" t="n">
-        <v>13.79</v>
+        <v>13.89</v>
       </c>
     </row>
   </sheetData>
@@ -3415,16 +3415,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3365</v>
+        <v>3432</v>
       </c>
       <c r="C12" t="n">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="D12" t="n">
-        <v>22877</v>
+        <v>23766</v>
       </c>
       <c r="E12" t="n">
-        <v>44.55</v>
+        <v>43.94</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4039,13 +4039,13 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D12" t="n">
-        <v>71.31999999999999</v>
+        <v>72.26000000000001</v>
       </c>
       <c r="E12" t="n">
-        <v>1.97</v>
+        <v>1.93</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -4063,17 +4063,17 @@
         </is>
       </c>
       <c r="I12" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J12" t="n">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="K12" t="n">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="L12" s="10" t="inlineStr">
         <is>
-          <t>missing-function-docstring: 39; trailing-whitespace: 26; no-member: 16; unexpected-keyword-arg: 16; broad-exception-caught: 11; 6/5: 10; 104/100: 7; undefined-variable: 6; protected-access: 5; 106/100: 4</t>
+          <t>missing-function-docstring: 39; trailing-whitespace: 32; no-member: 16; unexpected-keyword-arg: 16; broad-exception-caught: 11; 6/5: 10; 104/100: 7; undefined-variable: 6; 106/100: 5; protected-access: 5</t>
         </is>
       </c>
     </row>

</xml_diff>